<commit_message>
docs: update functional requirements, test case excels and coverage docs for heartbeat, watchdog and DeepSeek API
</commit_message>
<xml_diff>
--- a/Phytium_PPE_System_SourceCode/03_系统测试蚆盖分析报告_终稿.xlsx
+++ b/Phytium_PPE_System_SourceCode/03_系统测试蚆盖分析报告_终稿.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -794,6 +794,33 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>REQ-14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>DeepSeek AI 智能安全顾问</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>TC-11</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: adjust test cases and requirement sheets to establish a strict 1-to-1 mapping (TC-01~TC-14 to REQ-01~REQ-14)
</commit_message>
<xml_diff>
--- a/Phytium_PPE_System_SourceCode/03_系统测试蚆盖分析报告_终稿.xlsx
+++ b/Phytium_PPE_System_SourceCode/03_系统测试蚆盖分析报告_终稿.xlsx
@@ -17,13 +17,22 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +43,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +51,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,405 +441,405 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>功能项</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>测试编号</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>执行结果记录</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>测试蚆盖度</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>REQ-01</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>视频流采集</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>USB摄像头实时拉流</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>TC-01</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>REQ-02</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>模型推理（YOLOv5/v8）</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>视频源无感热切换</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>TC-02</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>REQ-03</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>安全帽乩戴检测</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>多线程无锁数据传输</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>TC-03</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>REQ-04</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>反光衣穿着检测</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>PPE 八类目标检测</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>REQ-05</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>未穿戴行为报警</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>复杂遮挡目标追踪</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>TC-05</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>REQ-06</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>UI 界面展示</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>违规报警物理阻断</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>TC-06</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>REQ-07</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>火焰/烟雾传感器采集</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>灾害环境硬中断报警</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>TC-07</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>REQ-08</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>外设联动（蜂鸣器/风扇）</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>零拷贝监控大屏</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>TC-08</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>REQ-09</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>主从核通信 (RPMsg)</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>硬件状态自视看板</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>TC-09</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>REQ-10</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>违规抓拍与本地存储</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>违规异步抓拍落盘</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>TC-10</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>REQ-11</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>嵌盘防洪机制</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>磁盘防洪自清洁机制</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>TC-11</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>REQ-12</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>主核心跳监控</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>主从核心跳通信</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>TC-12</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>REQ-13</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>看门狗(WDT)容错与告警</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>看门狗(WDT)容错与自愈</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>TC-13</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>REQ-14</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>DeepSeek AI 智能安全顾问</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>TC-11</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>DeepSeek AI 安全整改建议</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>TC-14</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>100%</t>
         </is>

</xml_diff>

<commit_message>
style: adjust excel row heights and column widths dynamically to prevent text truncation
</commit_message>
<xml_diff>
--- a/Phytium_PPE_System_SourceCode/03_系统测试蚆盖分析报告_终稿.xlsx
+++ b/Phytium_PPE_System_SourceCode/03_系统测试蚆盖分析报告_终稿.xlsx
@@ -439,8 +439,15 @@
   </sheetPr>
   <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="29" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
@@ -467,7 +474,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="29" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>REQ-01</t>
@@ -494,7 +501,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="29" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>REQ-02</t>
@@ -521,7 +528,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="29" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>REQ-03</t>
@@ -548,7 +555,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="29" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>REQ-04</t>
@@ -575,7 +582,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="29" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>REQ-05</t>
@@ -602,7 +609,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="29" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>REQ-06</t>
@@ -629,7 +636,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="29" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>REQ-07</t>
@@ -656,7 +663,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="29" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>REQ-08</t>
@@ -683,7 +690,7 @@
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="29" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>REQ-09</t>
@@ -710,7 +717,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="29" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>REQ-10</t>
@@ -737,7 +744,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="29" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>REQ-11</t>
@@ -764,7 +771,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="29" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>REQ-12</t>
@@ -791,7 +798,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="29" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>REQ-13</t>
@@ -818,7 +825,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="29" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>REQ-14</t>

</xml_diff>